<commit_message>
Présentation des taux en conformité avec la description dans le texte
Au lieu de calculer un taux des lits d'hôpital par habitant·e, calculer un taux d'habitant·e par lit
</commit_message>
<xml_diff>
--- a/Lits d'hôpital - DROM.xlsx
+++ b/Lits d'hôpital - DROM.xlsx
@@ -1,25 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rehl\Box\0FR - Equipe PIC\Adaptation juste\Projets\Santé et climat\Calculs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2170523231234/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32866766-BF5F-4726-8FBD-D7720481C816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F551E61-2F43-494D-808D-522555319623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="21600" windowHeight="11295" xr2:uid="{0FA5FE41-A271-4FA6-AEAC-1D642E1EBBCE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0FA5FE41-A271-4FA6-AEAC-1D642E1EBBCE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Offre hospitalière" sheetId="1" r:id="rId1"/>
-    <sheet name="Population par département" sheetId="2" r:id="rId2"/>
-    <sheet name="Taux lits par habitant·e" sheetId="3" r:id="rId3"/>
+    <sheet name="Taux lits par habitant·e" sheetId="3" r:id="rId1"/>
+    <sheet name="Offre hospitalière" sheetId="1" r:id="rId2"/>
+    <sheet name="Population par département" sheetId="2" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId4"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -85,19 +82,19 @@
     <t>Nombre d'habitants</t>
   </si>
   <si>
-    <t>Offre total</t>
-  </si>
-  <si>
     <t>Taux lits</t>
   </si>
   <si>
-    <t>Taux places</t>
-  </si>
-  <si>
-    <t>Taux total offre hospitalière</t>
-  </si>
-  <si>
     <t>Ensemble de tous les départements</t>
+  </si>
+  <si>
+    <t>Offre lits &amp; places</t>
+  </si>
+  <si>
+    <t>Offre lits</t>
+  </si>
+  <si>
+    <t>Lits par habitant·e</t>
   </si>
 </sst>
 </file>
@@ -175,198 +172,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Données offre hospitalier"/>
-      <sheetName val="Données population"/>
-      <sheetName val="Taux d'offre par habitant·e"/>
-      <sheetName val="Sources"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="2">
-          <cell r="B2">
-            <v>1095</v>
-          </cell>
-          <cell r="C2">
-            <v>275</v>
-          </cell>
-          <cell r="D2">
-            <v>763</v>
-          </cell>
-          <cell r="E2">
-            <v>128</v>
-          </cell>
-          <cell r="F2">
-            <v>235</v>
-          </cell>
-          <cell r="G2">
-            <v>193</v>
-          </cell>
-          <cell r="H2">
-            <v>201</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="B3">
-            <v>879</v>
-          </cell>
-          <cell r="C3">
-            <v>279</v>
-          </cell>
-          <cell r="D3">
-            <v>566</v>
-          </cell>
-          <cell r="E3">
-            <v>103</v>
-          </cell>
-          <cell r="F3">
-            <v>165</v>
-          </cell>
-          <cell r="G3">
-            <v>90</v>
-          </cell>
-          <cell r="H3">
-            <v>75</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="B4">
-            <v>722</v>
-          </cell>
-          <cell r="C4">
-            <v>71</v>
-          </cell>
-          <cell r="D4">
-            <v>127</v>
-          </cell>
-          <cell r="E4">
-            <v>30</v>
-          </cell>
-          <cell r="F4">
-            <v>94</v>
-          </cell>
-          <cell r="G4">
-            <v>42</v>
-          </cell>
-          <cell r="H4">
-            <v>89</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="B5">
-            <v>2186</v>
-          </cell>
-          <cell r="C5">
-            <v>540</v>
-          </cell>
-          <cell r="D5">
-            <v>953</v>
-          </cell>
-          <cell r="E5">
-            <v>82</v>
-          </cell>
-          <cell r="F5">
-            <v>398</v>
-          </cell>
-          <cell r="G5">
-            <v>281</v>
-          </cell>
-          <cell r="H5">
-            <v>695</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="B6">
-            <v>404</v>
-          </cell>
-          <cell r="C6">
-            <v>10</v>
-          </cell>
-          <cell r="D6">
-            <v>50</v>
-          </cell>
-          <cell r="E6">
-            <v>0</v>
-          </cell>
-          <cell r="F6">
-            <v>36</v>
-          </cell>
-          <cell r="G6">
-            <v>0</v>
-          </cell>
-          <cell r="H6">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="B7">
-            <v>182279</v>
-          </cell>
-          <cell r="C7">
-            <v>50007</v>
-          </cell>
-          <cell r="D7">
-            <v>98908</v>
-          </cell>
-          <cell r="E7">
-            <v>28906</v>
-          </cell>
-          <cell r="F7">
-            <v>38008</v>
-          </cell>
-          <cell r="G7">
-            <v>29635</v>
-          </cell>
-          <cell r="H7">
-            <v>18229</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1">
-        <row r="2">
-          <cell r="B2">
-            <v>380387</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="B3">
-            <v>355459</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="B4">
-            <v>292354</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="B5">
-            <v>896175</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="B6">
-            <v>329282</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="B7">
-            <v>66351959</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -685,6 +490,178 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F44444D-916E-48C1-9105-113F6840E47E}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3">
+        <f>SUM('Offre hospitalière'!B2:H2)</f>
+        <v>2890</v>
+      </c>
+      <c r="C2">
+        <f>SUM('Offre hospitalière'!B2:E2)</f>
+        <v>2261</v>
+      </c>
+      <c r="D2">
+        <f>C2/'Population par département'!B2</f>
+        <v>5.943946559687897E-3</v>
+      </c>
+      <c r="E2">
+        <f>'Population par département'!B2/'Taux lits par habitant·e'!C2</f>
+        <v>168.23839009287926</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3">
+        <f>SUM('Offre hospitalière'!B3:H3)</f>
+        <v>2157</v>
+      </c>
+      <c r="C3">
+        <f>SUM('Offre hospitalière'!B3:E3)</f>
+        <v>1827</v>
+      </c>
+      <c r="D3">
+        <f>C3/'Population par département'!B3</f>
+        <v>5.1398332859767231E-3</v>
+      </c>
+      <c r="E3">
+        <f>'Population par département'!B3/'Taux lits par habitant·e'!C3</f>
+        <v>194.55883962780516</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3">
+        <f>SUM('Offre hospitalière'!B4:H4)</f>
+        <v>1175</v>
+      </c>
+      <c r="C4">
+        <f>SUM('Offre hospitalière'!B4:E4)</f>
+        <v>950</v>
+      </c>
+      <c r="D4">
+        <f>C4/'Population par département'!B4</f>
+        <v>3.2494852131320249E-3</v>
+      </c>
+      <c r="E4">
+        <f>'Population par département'!B4/'Taux lits par habitant·e'!C4</f>
+        <v>307.74105263157895</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="3">
+        <f>SUM('Offre hospitalière'!B5:H5)</f>
+        <v>5135</v>
+      </c>
+      <c r="C5">
+        <f>SUM('Offre hospitalière'!B5:E5)</f>
+        <v>3761</v>
+      </c>
+      <c r="D5">
+        <f>C5/'Population par département'!B5</f>
+        <v>4.1967249700114373E-3</v>
+      </c>
+      <c r="E5">
+        <f>'Population par département'!B5/'Taux lits par habitant·e'!C5</f>
+        <v>238.28104227599042</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="3">
+        <f>SUM('Offre hospitalière'!B6:H6)</f>
+        <v>505</v>
+      </c>
+      <c r="C6">
+        <f>SUM('Offre hospitalière'!B6:E6)</f>
+        <v>464</v>
+      </c>
+      <c r="D6">
+        <f>C6/'Population par département'!B6</f>
+        <v>1.4091265237698993E-3</v>
+      </c>
+      <c r="E6">
+        <f>'Population par département'!B6/'Taux lits par habitant·e'!C6</f>
+        <v>709.6594827586207</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3">
+        <f>SUM('Offre hospitalière'!B7:H7)</f>
+        <v>445972</v>
+      </c>
+      <c r="C7">
+        <f>SUM('Offre hospitalière'!B7:E7)</f>
+        <v>360100</v>
+      </c>
+      <c r="D7">
+        <f>C7/'Population par département'!B7</f>
+        <v>5.4271193409677629E-3</v>
+      </c>
+      <c r="E7">
+        <f>'Population par département'!B7/'Taux lits par habitant·e'!C7</f>
+        <v>184.25981394057206</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="3">
+        <f>SUM(B2:B7)</f>
+        <v>457834</v>
+      </c>
+      <c r="C8">
+        <f>SUM(C2:C7)</f>
+        <v>369363</v>
+      </c>
+      <c r="D8">
+        <f>C8/SUM('Population par département'!B2:B7)</f>
+        <v>5.3838595370967884E-3</v>
+      </c>
+      <c r="E8">
+        <f>SUM('Population par département'!B2:B7)/'Taux lits par habitant·e'!C8</f>
+        <v>185.74035840081439</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FA00E16-DEA6-4602-A49B-612477F09121}">
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -874,18 +851,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9F51AD9-5861-4249-BEF5-3D2348AC0401}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -893,7 +870,7 @@
         <v>380387</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -901,7 +878,7 @@
         <v>355459</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -909,7 +886,7 @@
         <v>292354</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -917,7 +894,7 @@
         <v>896175</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -925,7 +902,7 @@
         <v>329282</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -933,177 +910,8 @@
         <v>66351959</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F44444D-916E-48C1-9105-113F6840E47E}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="3">
-        <f>SUM('[1]Données offre hospitalier'!B2:H2)</f>
-        <v>2890</v>
-      </c>
-      <c r="C2">
-        <f>SUM('[1]Données offre hospitalier'!B2:E2)/'[1]Données population'!B2</f>
-        <v>5.943946559687897E-3</v>
-      </c>
-      <c r="D2">
-        <f>SUM('[1]Données offre hospitalier'!F2:H2)/'[1]Données population'!B2</f>
-        <v>1.6535791181086631E-3</v>
-      </c>
-      <c r="E2">
-        <f>B2/'[1]Données population'!B2</f>
-        <v>7.5975256777965601E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="3">
-        <f>SUM('[1]Données offre hospitalier'!B3:H3)</f>
-        <v>2157</v>
-      </c>
-      <c r="C3">
-        <f>SUM('[1]Données offre hospitalier'!B3:E3)/'[1]Données population'!B3</f>
-        <v>5.1398332859767231E-3</v>
-      </c>
-      <c r="D3">
-        <f>SUM('[1]Données offre hospitalier'!F3:H3)/'[1]Données population'!B3</f>
-        <v>9.2837711240958878E-4</v>
-      </c>
-      <c r="E3">
-        <f>B3/'[1]Données population'!B3</f>
-        <v>6.0682103983863119E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="3">
-        <f>SUM('[1]Données offre hospitalier'!B4:H4)</f>
-        <v>1175</v>
-      </c>
-      <c r="C4">
-        <f>SUM('[1]Données offre hospitalier'!B4:E4)/'[1]Données population'!B4</f>
-        <v>3.2494852131320249E-3</v>
-      </c>
-      <c r="D4">
-        <f>SUM('[1]Données offre hospitalier'!F4:H4)/'[1]Données population'!B4</f>
-        <v>7.6961491889969012E-4</v>
-      </c>
-      <c r="E4">
-        <f>B4/'[1]Données population'!B4</f>
-        <v>4.0191001320317148E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="3">
-        <f>SUM('[1]Données offre hospitalier'!B5:H5)</f>
-        <v>5135</v>
-      </c>
-      <c r="C5">
-        <f>SUM('[1]Données offre hospitalier'!B5:E5)/'[1]Données population'!B5</f>
-        <v>4.1967249700114373E-3</v>
-      </c>
-      <c r="D5">
-        <f>SUM('[1]Données offre hospitalier'!F5:H5)/'[1]Données population'!B5</f>
-        <v>1.5331826931123944E-3</v>
-      </c>
-      <c r="E5">
-        <f>B5/'[1]Données population'!B5</f>
-        <v>5.7299076631238321E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="3">
-        <f>SUM('[1]Données offre hospitalier'!B6:H6)</f>
-        <v>505</v>
-      </c>
-      <c r="C6">
-        <f>SUM('[1]Données offre hospitalier'!B6:E6)/'[1]Données population'!B6</f>
-        <v>1.4091265237698993E-3</v>
-      </c>
-      <c r="D6">
-        <f>SUM('[1]Données offre hospitalier'!F6:H6)/'[1]Données population'!B6</f>
-        <v>1.2451333507449542E-4</v>
-      </c>
-      <c r="E6">
-        <f>B6/'[1]Données population'!B6</f>
-        <v>1.5336398588443947E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="3">
-        <f>SUM('[1]Données offre hospitalier'!B7:H7)</f>
-        <v>445972</v>
-      </c>
-      <c r="C7">
-        <f>SUM('[1]Données offre hospitalier'!B7:E7)/'[1]Données population'!B7</f>
-        <v>5.4271193409677629E-3</v>
-      </c>
-      <c r="D7">
-        <f>SUM('[1]Données offre hospitalier'!F7:H7)/'[1]Données population'!B7</f>
-        <v>1.2941893697516905E-3</v>
-      </c>
-      <c r="E7">
-        <f>B7/'[1]Données population'!B7</f>
-        <v>6.7213087107194525E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="2">
-        <f>SUM(B2:B7)</f>
-        <v>457834</v>
-      </c>
-      <c r="C8">
-        <f>(SUM('[1]Données offre hospitalier'!B2:E7)/(SUM('[1]Données population'!B2:B7)))</f>
-        <v>5.3838595370967884E-3</v>
-      </c>
-      <c r="D8">
-        <f>(SUM('[1]Données offre hospitalier'!F2:H7)/SUM('[1]Données population'!B2:B7))</f>
-        <v>1.2895591521253887E-3</v>
-      </c>
-      <c r="E8">
-        <f>(SUM('[1]Données offre hospitalier'!B2:H7)/SUM('[1]Données population'!B2:B7))</f>
-        <v>6.6734186892221771E-3</v>
-      </c>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F14" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>